<commit_message>
Add anti_symmetric notebook; update long_peptide
Add anti_symmetric comp_anti_symmetric.ipynb and its compiled bytecode. Update long_peptide package: add internal.py, annot_diff_test.xlsx, protein_result.csv and temporary Excel artifacts; modify annot.py, line_finding.py, notebooks (analysis.ipynb, deiso.ipynb) and protein.csv. Also update .DS_Store entries.
</commit_message>
<xml_diff>
--- a/long_peptide/isocolumn.xlsx
+++ b/long_peptide/isocolumn.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinmbp/Desktop/2D_spec_dict/long_peptide/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D886E19-9F3D-664D-83B1-1F988EC39EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBD11F4C-6210-9A40-AC3A-28BB2162860A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="57600" windowHeight="32400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22400" yWindow="500" windowWidth="28800" windowHeight="26680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3+" sheetId="3" r:id="rId1"/>
@@ -2451,10 +2451,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AF41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="32" width="44.5" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="32.83203125" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:32">
       <c r="A1" s="1" t="s">

</xml_diff>